<commit_message>
Wording fixes (thresholds, permutation, independently generated screens); recheck of zero-record PubMed pairs
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/figures/supporting_information/S8_Table.xlsx
+++ b/figures/supporting_information/S8_Table.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PubMed counts per pair" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DGIdb per gene" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recheck of zero-record pairs" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3888,4 +3889,372 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Symbol</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Lineage</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>pubmed_records_with_aliases</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>titles_of_returned_records</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>TUBB4B</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ampulla of vater</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>NHLRC2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>thyroid</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>DCAF7</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>myeloid</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>UMPS</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>lymphoid</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>SEPHS2</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>kidney</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>ADSL</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>myeloid</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>CDAN1</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>lymphoid</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>ADSL</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>lymphoid</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Metabolic pathways for the activation of the antiretroviral agent 2',3'-dideoxyadenosine in human lymphoid cells.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>SNAP23</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>pleura</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>WDR36</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>myeloid</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>FERMT2</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>soft tissue</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>A suppressive role of mitogen inducible gene-2 in mesenchymal cancer cell invasion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>FAM50A</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>lymphoid</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>FAM50A</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>bladder/urinary tract</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>FERMT2</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>pleura</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>INTS6</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>skin</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>AP2S1</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>myeloid</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>CTPS1</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>myeloid</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>CDAN1</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>myeloid</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>ELOB</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>cervix</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>FERMT2</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>ovary/fallopian tube</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Effects of Smad3 on the proliferation and steroidogenesis in human ovarian luteinized granulosa cells.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>